<commit_message>
Fix Chrome headless configuration for CI/CD - Add intelligent CI detection and Chrome setup in GitHub Actions
</commit_message>
<xml_diff>
--- a/test output/ExcelReport/ExtentExcel.xlsx
+++ b/test output/ExcelReport/ExtentExcel.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="64">
   <si>
     <t>Duration</t>
   </si>
@@ -189,16 +189,16 @@
     <t>device</t>
   </si>
   <si>
-    <t>Sep 12, 2025 6:15:47 PM</t>
+    <t>Sep 12, 2025 6:33:31 PM</t>
   </si>
   <si>
-    <t>Sep 12, 2025 6:10:06 PM</t>
+    <t>Sep 12, 2025 6:32:10 PM</t>
   </si>
   <si>
-    <t>Sep 12, 2025 6:15:43 PM</t>
+    <t>Sep 12, 2025 6:33:26 PM</t>
   </si>
   <si>
-    <t>5 m 37.093 s</t>
+    <t>1 m 16.092 s</t>
   </si>
   <si>
     <t>100%</t>
@@ -207,7 +207,7 @@
     <t>searching for a product</t>
   </si>
   <si>
-    <t>1 m 5.417 s</t>
+    <t>40.750 s</t>
   </si>
   <si>
     <t>Searching on BestBuy</t>
@@ -216,52 +216,7 @@
     <t>adding product to cart</t>
   </si>
   <si>
-    <t>37.473 s</t>
-  </si>
-  <si>
-    <t>checking product is in the cart page</t>
-  </si>
-  <si>
-    <t>33.216 s</t>
-  </si>
-  <si>
-    <t>Remove item from cart</t>
-  </si>
-  <si>
-    <t>4.516 s</t>
-  </si>
-  <si>
-    <t>Password Validations</t>
-  </si>
-  <si>
-    <t>23.695 s</t>
-  </si>
-  <si>
-    <t>User operations on BestBuy</t>
-  </si>
-  <si>
-    <t>24.608 s</t>
-  </si>
-  <si>
-    <t>29.998 s</t>
-  </si>
-  <si>
-    <t>Successfully register a new Staples user</t>
-  </si>
-  <si>
-    <t>1 m 8.095 s</t>
-  </si>
-  <si>
-    <t>Negative Test - Incorrect phone number format on Staples</t>
-  </si>
-  <si>
-    <t>30.027 s</t>
-  </si>
-  <si>
-    <t>Clean up</t>
-  </si>
-  <si>
-    <t>17.538 s</t>
+    <t>34.081 s</t>
   </si>
   <si>
     <t>@Positive</t>
@@ -273,43 +228,7 @@
     <t>@UC-102</t>
   </si>
   <si>
-    <t>@UC-103</t>
-  </si>
-  <si>
-    <t>@UC-104</t>
-  </si>
-  <si>
-    <t>@UC-105</t>
-  </si>
-  <si>
-    <t>@PasswordValidation</t>
-  </si>
-  <si>
-    <t>@UC-106</t>
-  </si>
-  <si>
-    <t>@Negative</t>
-  </si>
-  <si>
-    <t>@UC-107</t>
-  </si>
-  <si>
-    <t>@Login</t>
-  </si>
-  <si>
-    <t>@UC-108</t>
-  </si>
-  <si>
-    <t>@phoneValidation</t>
-  </si>
-  <si>
-    <t>@UC-109</t>
-  </si>
-  <si>
-    <t>2 m 20.743 s</t>
-  </si>
-  <si>
-    <t>3 m 14.067 s</t>
+    <t>1 m 14.867 s</t>
   </si>
 </sst>
 </file>
@@ -1877,76 +1796,28 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22:$B$31</c:f>
+              <c:f>Scenarios!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>searching for a product</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>adding product to cart</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>checking product is in the cart page</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Remove item from cart</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Successfully register a new Staples user</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Negative Test - Incorrect phone number format on Staples</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Clean up</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$H$22:$H$31</c:f>
+              <c:f>Scenarios!$H$22:$H$23</c:f>
               <c:numCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>3.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>3.0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3.0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3.0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>6.0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6.0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6.0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>9.0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>6.0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2003,45 +1874,21 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22:$B$31</c:f>
+              <c:f>Scenarios!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>searching for a product</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>adding product to cart</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>checking product is in the cart page</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Remove item from cart</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Successfully register a new Staples user</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Negative Test - Incorrect phone number format on Staples</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Clean up</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$J$22:$J$31</c:f>
+              <c:f>Scenarios!$J$22:$J$23</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2097,45 +1944,21 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22:$B$31</c:f>
+              <c:f>Scenarios!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>searching for a product</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>adding product to cart</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>checking product is in the cart page</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Remove item from cart</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Password Validations</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Successfully register a new Staples user</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Negative Test - Incorrect phone number format on Staples</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Clean up</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$I$22:$I$31</c:f>
+              <c:f>Scenarios!$I$22:$I$23</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2531,9 +2354,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Tags!$B$22:$B$35</c:f>
+              <c:f>Tags!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="14"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>@Positive</c:v>
                 </c:pt>
@@ -2542,88 +2365,22 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>@UC-102</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>@UC-103</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>@UC-104</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>@UC-105</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>@PasswordValidation</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>@UC-106</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>@Negative</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>@UC-107</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>@Login</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>@UC-108</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>@phoneValidation</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>@UC-109</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tags!$D$22:$D$35</c:f>
+              <c:f>Tags!$D$22:$D$24</c:f>
               <c:numCache>
-                <c:ptCount val="14"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>8.0</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2.0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>3.0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>2.0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.0</c:v>
-                </c:pt>
-                <c:pt idx="13">
                   <c:v>1.0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2682,9 +2439,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Tags!$B$22:$B$35</c:f>
+              <c:f>Tags!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="14"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>@Positive</c:v>
                 </c:pt>
@@ -2693,46 +2450,13 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>@UC-102</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>@UC-103</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>@UC-104</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>@UC-105</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>@PasswordValidation</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>@UC-106</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>@Negative</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>@UC-107</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>@Login</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>@UC-108</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>@phoneValidation</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>@UC-109</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tags!$F$22:$F$35</c:f>
+              <c:f>Tags!$F$22:$F$24</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2789,9 +2513,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Tags!$B$22:$B$35</c:f>
+              <c:f>Tags!$B$22:$B$24</c:f>
               <c:strCache>
-                <c:ptCount val="14"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>@Positive</c:v>
                 </c:pt>
@@ -2800,46 +2524,13 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>@UC-102</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>@UC-103</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>@UC-104</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>@UC-105</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>@PasswordValidation</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>@UC-106</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>@Negative</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>@UC-107</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>@Login</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>@UC-108</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>@phoneValidation</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>@UC-109</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tags!$E$22:$E$35</c:f>
+              <c:f>Tags!$E$22:$E$24</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -3044,28 +2735,22 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Features!$B$22:$B$23</c:f>
+              <c:f>Features!$B$22</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Searching on BestBuy</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>User operations on BestBuy</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Features!$F$22:$F$23</c:f>
+              <c:f>Features!$F$22</c:f>
               <c:numCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>4.0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>6.0</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3122,21 +2807,18 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Features!$B$22:$B$23</c:f>
+              <c:f>Features!$B$22</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Searching on BestBuy</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>User operations on BestBuy</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Features!$H$22:$H$23</c:f>
+              <c:f>Features!$H$22</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -3192,21 +2874,18 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Features!$B$22:$B$23</c:f>
+              <c:f>Features!$B$22</c:f>
               <c:strCache>
-                <c:ptCount val="2"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>Searching on BestBuy</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>User operations on BestBuy</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Features!$G$22:$G$23</c:f>
+              <c:f>Features!$G$22</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -6139,7 +5818,7 @@
     <col min="7" max="7" customWidth="true" width="20.85546875"/>
   </cols>
   <sheetData/>
-  <sheetProtection sheet="true" password="F4D3" scenarios="true" objects="true"/>
+  <sheetProtection sheet="true" password="9155" scenarios="true" objects="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -6148,7 +5827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B20:J31"/>
+  <dimension ref="B20:J23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="1.42578125"/>
@@ -6255,206 +5934,6 @@
       </c>
       <c r="I23" s="59"/>
       <c r="J23" s="60"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="54" t="s">
-        <v>60</v>
-      </c>
-      <c r="C24" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="56" t="s">
-        <v>61</v>
-      </c>
-      <c r="E24" s="54" t="s">
-        <v>57</v>
-      </c>
-      <c r="F24" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G24" s="57" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="H24" s="58" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="I24" s="59"/>
-      <c r="J24" s="60"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="C25" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" s="56" t="s">
-        <v>63</v>
-      </c>
-      <c r="E25" s="54" t="s">
-        <v>57</v>
-      </c>
-      <c r="F25" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G25" s="57" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="H25" s="58" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="I25" s="59"/>
-      <c r="J25" s="60"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="54" t="s">
-        <v>64</v>
-      </c>
-      <c r="C26" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="56" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="F26" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G26" s="57" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="H26" s="58" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="I26" s="59"/>
-      <c r="J26" s="60"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="54" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D27" s="56" t="s">
-        <v>67</v>
-      </c>
-      <c r="E27" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="F27" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G27" s="57" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="H27" s="58" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="I27" s="59"/>
-      <c r="J27" s="60"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="54" t="s">
-        <v>64</v>
-      </c>
-      <c r="C28" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D28" s="56" t="s">
-        <v>68</v>
-      </c>
-      <c r="E28" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="F28" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G28" s="57" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="H28" s="58" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="I28" s="59"/>
-      <c r="J28" s="60"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="54" t="s">
-        <v>69</v>
-      </c>
-      <c r="C29" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D29" s="56" t="s">
-        <v>70</v>
-      </c>
-      <c r="E29" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="F29" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G29" s="57" t="n">
-        <v>9.0</v>
-      </c>
-      <c r="H29" s="58" t="n">
-        <v>9.0</v>
-      </c>
-      <c r="I29" s="59"/>
-      <c r="J29" s="60"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="54" t="s">
-        <v>71</v>
-      </c>
-      <c r="C30" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D30" s="56" t="s">
-        <v>72</v>
-      </c>
-      <c r="E30" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="F30" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G30" s="57" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="H30" s="58" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="I30" s="59"/>
-      <c r="J30" s="60"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="54" t="s">
-        <v>73</v>
-      </c>
-      <c r="C31" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D31" s="56" t="s">
-        <v>74</v>
-      </c>
-      <c r="E31" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="F31" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G31" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="H31" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="I31" s="59"/>
-      <c r="J31" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6470,7 +5949,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B20:I64"/>
+  <dimension ref="B20:I32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="1.28515625"/>
@@ -6512,13 +5991,13 @@
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s" s="54">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C22" s="57" t="n">
-        <v>8.0</v>
+        <v>2.0</v>
       </c>
       <c r="D22" s="58" t="n">
-        <v>8.0</v>
+        <v>2.0</v>
       </c>
       <c r="E22" s="59"/>
       <c r="F22" s="60"/>
@@ -6528,7 +6007,7 @@
     </row>
     <row r="23">
       <c r="B23" s="54" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C23" s="57" t="n">
         <v>1.0</v>
@@ -6544,7 +6023,7 @@
     </row>
     <row r="24">
       <c r="B24" s="54" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C24" s="57" t="n">
         <v>1.0</v>
@@ -6558,632 +6037,101 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="54" t="s">
-        <v>78</v>
-      </c>
-      <c r="C25" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D25" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E25" s="59"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="61" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="54" t="s">
-        <v>79</v>
-      </c>
-      <c r="C26" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D26" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E26" s="59"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="61" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="54" t="s">
-        <v>80</v>
-      </c>
-      <c r="C27" s="57" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="D27" s="58" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="E27" s="59"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="61" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="54" t="s">
-        <v>81</v>
-      </c>
-      <c r="C28" s="57" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="D28" s="58" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="E28" s="59"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="61" t="s">
-        <v>54</v>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28" s="35" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="54" t="s">
-        <v>82</v>
-      </c>
-      <c r="C29" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D29" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E29" s="59"/>
-      <c r="F29" s="60"/>
-      <c r="G29" s="61" t="s">
-        <v>54</v>
+        <v>60</v>
+      </c>
+      <c r="C29" s="62" t="s">
+        <v>57</v>
+      </c>
+      <c r="D29" s="53"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="53"/>
+      <c r="G29" s="53"/>
+      <c r="H29" s="62" t="s">
+        <v>55</v>
+      </c>
+      <c r="I29" s="55" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="54" t="s">
-        <v>83</v>
-      </c>
-      <c r="C30" s="57" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="D30" s="58" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="E30" s="59"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="61" t="s">
-        <v>54</v>
+      <c r="B30" s="53"/>
+      <c r="C30" s="53"/>
+      <c r="D30" s="53"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="53"/>
+      <c r="G30" s="53"/>
+      <c r="H30" s="62" t="s">
+        <v>58</v>
+      </c>
+      <c r="I30" s="55" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="54" t="s">
-        <v>84</v>
-      </c>
-      <c r="C31" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D31" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E31" s="59"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="61" t="s">
-        <v>54</v>
+        <v>61</v>
+      </c>
+      <c r="C31" s="62" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="53"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="53"/>
+      <c r="G31" s="53"/>
+      <c r="H31" s="62" t="s">
+        <v>55</v>
+      </c>
+      <c r="I31" s="55" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="54" t="s">
-        <v>85</v>
-      </c>
-      <c r="C32" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D32" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E32" s="59"/>
-      <c r="F32" s="60"/>
-      <c r="G32" s="61" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="C33" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D33" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E33" s="59"/>
-      <c r="F33" s="60"/>
-      <c r="G33" s="61" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="54" t="s">
-        <v>87</v>
-      </c>
-      <c r="C34" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D34" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E34" s="59"/>
-      <c r="F34" s="60"/>
-      <c r="G34" s="61" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="54" t="s">
-        <v>88</v>
-      </c>
-      <c r="C35" s="57" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="D35" s="58" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="E35" s="59"/>
-      <c r="F35" s="60"/>
-      <c r="G35" s="61" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="35" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" s="49" t="s">
-        <v>16</v>
-      </c>
-      <c r="D39" s="49"/>
-      <c r="E39" s="49"/>
-      <c r="F39" s="49"/>
-      <c r="G39" s="49"/>
-      <c r="H39" s="36" t="s">
-        <v>17</v>
-      </c>
-      <c r="I39" s="35" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="54" t="s">
-        <v>75</v>
-      </c>
-      <c r="C40" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="62" t="s">
         <v>57</v>
       </c>
-      <c r="D40" s="53"/>
-      <c r="E40" s="53"/>
-      <c r="F40" s="53"/>
-      <c r="G40" s="53"/>
-      <c r="H40" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="I40" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="53"/>
-      <c r="C41" s="53"/>
-      <c r="D41" s="53"/>
-      <c r="E41" s="53"/>
-      <c r="F41" s="53"/>
-      <c r="G41" s="53"/>
-      <c r="H41" s="62" t="s">
+      <c r="D32" s="53"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53"/>
+      <c r="G32" s="53"/>
+      <c r="H32" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="I41" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="53"/>
-      <c r="C42" s="53"/>
-      <c r="D42" s="53"/>
-      <c r="E42" s="53"/>
-      <c r="F42" s="53"/>
-      <c r="G42" s="53"/>
-      <c r="H42" s="62" t="s">
-        <v>60</v>
-      </c>
-      <c r="I42" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="53"/>
-      <c r="C43" s="53"/>
-      <c r="D43" s="53"/>
-      <c r="E43" s="53"/>
-      <c r="F43" s="53"/>
-      <c r="G43" s="53"/>
-      <c r="H43" s="62" t="s">
-        <v>62</v>
-      </c>
-      <c r="I43" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="53"/>
-      <c r="C44" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D44" s="53"/>
-      <c r="E44" s="53"/>
-      <c r="F44" s="53"/>
-      <c r="G44" s="53"/>
-      <c r="H44" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I44" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="53"/>
-      <c r="C45" s="53"/>
-      <c r="D45" s="53"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="53"/>
-      <c r="G45" s="53"/>
-      <c r="H45" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I45" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="53"/>
-      <c r="C46" s="53"/>
-      <c r="D46" s="53"/>
-      <c r="E46" s="53"/>
-      <c r="F46" s="53"/>
-      <c r="G46" s="53"/>
-      <c r="H46" s="62" t="s">
-        <v>69</v>
-      </c>
-      <c r="I46" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="53"/>
-      <c r="C47" s="53"/>
-      <c r="D47" s="53"/>
-      <c r="E47" s="53"/>
-      <c r="F47" s="53"/>
-      <c r="G47" s="53"/>
-      <c r="H47" s="62" t="s">
-        <v>73</v>
-      </c>
-      <c r="I47" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="54" t="s">
-        <v>76</v>
-      </c>
-      <c r="C48" s="62" t="s">
-        <v>57</v>
-      </c>
-      <c r="D48" s="53"/>
-      <c r="E48" s="53"/>
-      <c r="F48" s="53"/>
-      <c r="G48" s="53"/>
-      <c r="H48" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="I48" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="54" t="s">
-        <v>77</v>
-      </c>
-      <c r="C49" s="62" t="s">
-        <v>57</v>
-      </c>
-      <c r="D49" s="53"/>
-      <c r="E49" s="53"/>
-      <c r="F49" s="53"/>
-      <c r="G49" s="53"/>
-      <c r="H49" s="62" t="s">
-        <v>58</v>
-      </c>
-      <c r="I49" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="54" t="s">
-        <v>78</v>
-      </c>
-      <c r="C50" s="62" t="s">
-        <v>57</v>
-      </c>
-      <c r="D50" s="53"/>
-      <c r="E50" s="53"/>
-      <c r="F50" s="53"/>
-      <c r="G50" s="53"/>
-      <c r="H50" s="62" t="s">
-        <v>60</v>
-      </c>
-      <c r="I50" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="54" t="s">
-        <v>79</v>
-      </c>
-      <c r="C51" s="62" t="s">
-        <v>57</v>
-      </c>
-      <c r="D51" s="53"/>
-      <c r="E51" s="53"/>
-      <c r="F51" s="53"/>
-      <c r="G51" s="53"/>
-      <c r="H51" s="62" t="s">
-        <v>62</v>
-      </c>
-      <c r="I51" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="54" t="s">
-        <v>80</v>
-      </c>
-      <c r="C52" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D52" s="53"/>
-      <c r="E52" s="53"/>
-      <c r="F52" s="53"/>
-      <c r="G52" s="53"/>
-      <c r="H52" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I52" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="53"/>
-      <c r="C53" s="53"/>
-      <c r="D53" s="53"/>
-      <c r="E53" s="53"/>
-      <c r="F53" s="53"/>
-      <c r="G53" s="53"/>
-      <c r="H53" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I53" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="54" t="s">
-        <v>81</v>
-      </c>
-      <c r="C54" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D54" s="53"/>
-      <c r="E54" s="53"/>
-      <c r="F54" s="53"/>
-      <c r="G54" s="53"/>
-      <c r="H54" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I54" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="53"/>
-      <c r="C55" s="53"/>
-      <c r="D55" s="53"/>
-      <c r="E55" s="53"/>
-      <c r="F55" s="53"/>
-      <c r="G55" s="53"/>
-      <c r="H55" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I55" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="53"/>
-      <c r="C56" s="53"/>
-      <c r="D56" s="53"/>
-      <c r="E56" s="53"/>
-      <c r="F56" s="53"/>
-      <c r="G56" s="53"/>
-      <c r="H56" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I56" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="54" t="s">
-        <v>82</v>
-      </c>
-      <c r="C57" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D57" s="53"/>
-      <c r="E57" s="53"/>
-      <c r="F57" s="53"/>
-      <c r="G57" s="53"/>
-      <c r="H57" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I57" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="54" t="s">
-        <v>83</v>
-      </c>
-      <c r="C58" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D58" s="53"/>
-      <c r="E58" s="53"/>
-      <c r="F58" s="53"/>
-      <c r="G58" s="53"/>
-      <c r="H58" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="I58" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="53"/>
-      <c r="C59" s="53"/>
-      <c r="D59" s="53"/>
-      <c r="E59" s="53"/>
-      <c r="F59" s="53"/>
-      <c r="G59" s="53"/>
-      <c r="H59" s="62" t="s">
-        <v>71</v>
-      </c>
-      <c r="I59" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="54" t="s">
-        <v>84</v>
-      </c>
-      <c r="C60" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D60" s="53"/>
-      <c r="E60" s="53"/>
-      <c r="F60" s="53"/>
-      <c r="G60" s="53"/>
-      <c r="H60" s="62" t="s">
-        <v>69</v>
-      </c>
-      <c r="I60" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" s="54" t="s">
-        <v>85</v>
-      </c>
-      <c r="C61" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D61" s="53"/>
-      <c r="E61" s="53"/>
-      <c r="F61" s="53"/>
-      <c r="G61" s="53"/>
-      <c r="H61" s="62" t="s">
-        <v>69</v>
-      </c>
-      <c r="I61" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="C62" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D62" s="53"/>
-      <c r="E62" s="53"/>
-      <c r="F62" s="53"/>
-      <c r="G62" s="53"/>
-      <c r="H62" s="62" t="s">
-        <v>71</v>
-      </c>
-      <c r="I62" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="54" t="s">
-        <v>87</v>
-      </c>
-      <c r="C63" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D63" s="53"/>
-      <c r="E63" s="53"/>
-      <c r="F63" s="53"/>
-      <c r="G63" s="53"/>
-      <c r="H63" s="62" t="s">
-        <v>71</v>
-      </c>
-      <c r="I63" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="54" t="s">
-        <v>88</v>
-      </c>
-      <c r="C64" s="62" t="s">
-        <v>66</v>
-      </c>
-      <c r="D64" s="53"/>
-      <c r="E64" s="53"/>
-      <c r="F64" s="53"/>
-      <c r="G64" s="53"/>
-      <c r="H64" s="62" t="s">
-        <v>73</v>
-      </c>
-      <c r="I64" s="55" t="s">
+      <c r="I32" s="55" t="s">
         <v>29</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="8">
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="C20:G20"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="B40:B47"/>
-    <mergeCell ref="C40:G43"/>
-    <mergeCell ref="C44:G47"/>
-    <mergeCell ref="C48:G48"/>
-    <mergeCell ref="C49:G49"/>
-    <mergeCell ref="C50:G50"/>
-    <mergeCell ref="C51:G51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C52:G53"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="C54:G56"/>
-    <mergeCell ref="C57:G57"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:G59"/>
-    <mergeCell ref="C60:G60"/>
-    <mergeCell ref="C61:G61"/>
-    <mergeCell ref="C62:G62"/>
-    <mergeCell ref="C63:G63"/>
-    <mergeCell ref="C64:G64"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:G30"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C32:G32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7193,7 +6141,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B18:M23"/>
+  <dimension ref="B18:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="2.0"/>
@@ -7274,13 +6222,13 @@
         <v>29</v>
       </c>
       <c r="D22" s="56" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="E22" s="57" t="n">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="F22" s="58" t="n">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="G22" s="59"/>
       <c r="H22" s="60"/>
@@ -7288,43 +6236,13 @@
         <v>54</v>
       </c>
       <c r="J22" s="57" t="n">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="K22" s="58" t="n">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="L22" s="59"/>
       <c r="M22" s="60"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="54" t="s">
-        <v>66</v>
-      </c>
-      <c r="C23" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D23" s="56" t="s">
-        <v>90</v>
-      </c>
-      <c r="E23" s="57" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="F23" s="58" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="G23" s="59"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="61" t="s">
-        <v>54</v>
-      </c>
-      <c r="J23" s="57" t="n">
-        <v>34.0</v>
-      </c>
-      <c r="K23" s="58" t="n">
-        <v>34.0</v>
-      </c>
-      <c r="L23" s="59"/>
-      <c r="M23" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7383,19 +6301,19 @@
         <v>3</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>9</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>10.0</v>
+        <v>2.0</v>
       </c>
       <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="H2" t="n" s="0">
-        <v>46.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -7450,21 +6368,21 @@
       </c>
       <c r="D5" t="n" s="0">
         <f>SUM(D2:D4)</f>
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>20</v>
       </c>
       <c r="F5" t="n" s="0">
         <f>SUM(F2:F4)</f>
-        <v>10.0</v>
+        <v>2.0</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>21</v>
       </c>
       <c r="H5" t="n" s="0">
         <f>SUM(H2:H4)</f>
-        <v>46.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>